<commit_message>
Fixed UI code in QA env
</commit_message>
<xml_diff>
--- a/TestData/Excel/TC.XLSX
+++ b/TestData/Excel/TC.XLSX
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27040" windowHeight="10920"/>
+    <workbookView windowWidth="27040" windowHeight="9980"/>
   </bookViews>
   <sheets>
     <sheet name="TC" sheetId="2" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="210">
   <si>
     <t>Test ID</t>
   </si>
@@ -51,6 +51,12 @@
   </si>
   <si>
     <t>Expected Result</t>
+  </si>
+  <si>
+    <t>Actual Result</t>
+  </si>
+  <si>
+    <t>Status</t>
   </si>
   <si>
     <t>TC-001</t>
@@ -1906,13 +1912,14 @@
     <col min="6" max="6" width="35.8046875" customWidth="1"/>
     <col min="7" max="7" width="52.078125" customWidth="1"/>
     <col min="8" max="8" width="49.859375" customWidth="1"/>
+    <col min="9" max="9" width="12.2421875" customWidth="1"/>
     <col min="14" max="14" width="9.0625" customWidth="1"/>
     <col min="15" max="15" width="7.65625" customWidth="1"/>
     <col min="16" max="16" width="8.75" customWidth="1"/>
     <col min="17" max="17" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" spans="1:8">
+    <row r="1" ht="22" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1937,70 +1944,76 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="2" ht="17" spans="1:17">
       <c r="A2" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="N2" s="6" t="s">
         <v>1</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" ht="51" spans="1:17">
       <c r="A3" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="O3" s="7">
         <v>2</v>
@@ -2014,29 +2027,29 @@
     </row>
     <row r="4" ht="17" spans="1:17">
       <c r="A4" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="O4" s="7">
         <v>0</v>
@@ -2050,31 +2063,31 @@
     </row>
     <row r="5" ht="34" spans="1:17">
       <c r="A5" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="O5" s="7">
         <v>0</v>
@@ -2088,29 +2101,29 @@
     </row>
     <row r="6" ht="17" spans="1:17">
       <c r="A6" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="O6" s="7">
         <v>0</v>
@@ -2124,29 +2137,29 @@
     </row>
     <row r="7" ht="34" spans="1:17">
       <c r="A7" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="O7" s="7">
         <v>0</v>
@@ -2160,29 +2173,29 @@
     </row>
     <row r="8" ht="34" spans="1:17">
       <c r="A8" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="O8" s="7">
         <v>0</v>
@@ -2196,29 +2209,29 @@
     </row>
     <row r="9" ht="34" spans="1:17">
       <c r="A9" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="O9" s="7">
         <v>2</v>
@@ -2232,31 +2245,31 @@
     </row>
     <row r="10" ht="17" spans="1:17">
       <c r="A10" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="N10" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="O10" s="8">
         <v>4</v>
@@ -2270,778 +2283,778 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="H34" s="2" t="s">
         <v>170</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="36" spans="1:8">
       <c r="A36" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B36" s="5"/>
       <c r="C36" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="G36" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>176</v>
-      </c>
       <c r="H36" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="38" spans="1:8">
       <c r="A38" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B40" s="5"/>
       <c r="C40" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="41" spans="1:8">
       <c r="A41" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="42" spans="1:8">
       <c r="A42" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B42" s="5"/>
       <c r="C42" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modified Test Files according to Modulewise
</commit_message>
<xml_diff>
--- a/TestData/Excel/TC.XLSX
+++ b/TestData/Excel/TC.XLSX
@@ -65,7 +65,7 @@
     <t>Authentication and Login</t>
   </si>
   <si>
-    <t>Login through API</t>
+    <t>API login succeeds</t>
   </si>
   <si>
     <t>API</t>
@@ -95,7 +95,7 @@
     <t>TC-002</t>
   </si>
   <si>
-    <t>Login with Valid Credentials</t>
+    <t>Valid login opens home</t>
   </si>
   <si>
     <t>UI</t>
@@ -116,7 +116,7 @@
     <t>TC-003</t>
   </si>
   <si>
-    <t>Login with Invalid Credentials</t>
+    <t>Invalid login shows error</t>
   </si>
   <si>
     <t>Verify appropriate error for invalid credentials</t>
@@ -134,7 +134,7 @@
     <t>TC-004</t>
   </si>
   <si>
-    <t>Create Label</t>
+    <t>Create label</t>
   </si>
   <si>
     <t>Verify labels can be created successfully</t>
@@ -152,7 +152,7 @@
     <t>TC-005</t>
   </si>
   <si>
-    <t>Fetch Label API</t>
+    <t>Fetch labels</t>
   </si>
   <si>
     <t>GET</t>
@@ -170,7 +170,7 @@
     <t>TC-006</t>
   </si>
   <si>
-    <t>Fetch Label Usage API</t>
+    <t>Fetch label usage</t>
   </si>
   <si>
     <t>Verify label usage statistics can be fetched</t>
@@ -185,7 +185,7 @@
     <t>TC-007</t>
   </si>
   <si>
-    <t>Update Label</t>
+    <t>Update label</t>
   </si>
   <si>
     <t>PUT</t>
@@ -206,7 +206,7 @@
     <t>TC-008</t>
   </si>
   <si>
-    <t>Delete Label</t>
+    <t>Delete label</t>
   </si>
   <si>
     <t>DELETE</t>
@@ -227,7 +227,7 @@
     <t>TC-009</t>
   </si>
   <si>
-    <t>Opening Balance API</t>
+    <t>Fetch opening balance</t>
   </si>
   <si>
     <t>Verify opening balance can be retrieved</t>
@@ -242,7 +242,7 @@
     <t>TC-010</t>
   </si>
   <si>
-    <t>Create Debit Category</t>
+    <t>Create debit category</t>
   </si>
   <si>
     <t>Verify debit category can be created successfully</t>
@@ -257,7 +257,7 @@
     <t>TC-011</t>
   </si>
   <si>
-    <t>Fetch Categories</t>
+    <t>Fetch categories</t>
   </si>
   <si>
     <t>Verify all categories can be retrieved</t>
@@ -269,7 +269,7 @@
     <t>TC-012</t>
   </si>
   <si>
-    <t>Update Debit Category</t>
+    <t>Update debit category</t>
   </si>
   <si>
     <t>Verify debit category can be updated</t>
@@ -284,7 +284,7 @@
     <t>TC-013</t>
   </si>
   <si>
-    <t>Delete Debit Category</t>
+    <t>Delete debit category</t>
   </si>
   <si>
     <t>Verify debit category can be deleted</t>
@@ -299,7 +299,7 @@
     <t>TC-014</t>
   </si>
   <si>
-    <t>Create Credit Category</t>
+    <t>Create credit category</t>
   </si>
   <si>
     <t>Verify credit category can be created successfully</t>
@@ -311,7 +311,7 @@
     <t>TC-015</t>
   </si>
   <si>
-    <t>Update Credit Category</t>
+    <t>Update credit category</t>
   </si>
   <si>
     <t>Verify credit category can be updated</t>
@@ -323,7 +323,7 @@
     <t>TC-016</t>
   </si>
   <si>
-    <t>Delete Credit Category</t>
+    <t>Delete credit category</t>
   </si>
   <si>
     <t>Verify credit category can be deleted</t>
@@ -335,7 +335,7 @@
     <t>TC-017</t>
   </si>
   <si>
-    <t>Create Given Category</t>
+    <t>Create given category</t>
   </si>
   <si>
     <t>Verify given category can be created</t>
@@ -350,7 +350,7 @@
     <t>TC-018</t>
   </si>
   <si>
-    <t>Fetch Given Category</t>
+    <t>Fetch given category</t>
   </si>
   <si>
     <t>Verify given category can be retrieved</t>
@@ -365,7 +365,7 @@
     <t>TC-019</t>
   </si>
   <si>
-    <t>Update Given Category</t>
+    <t>Update given category</t>
   </si>
   <si>
     <t>Verify given category can be updated</t>
@@ -377,7 +377,7 @@
     <t>TC-020</t>
   </si>
   <si>
-    <t>Delete Given Category</t>
+    <t>Delete given category</t>
   </si>
   <si>
     <t>Verify given category can be deleted</t>
@@ -386,7 +386,7 @@
     <t>TC-021</t>
   </si>
   <si>
-    <t>Create Received Category</t>
+    <t>Create received category</t>
   </si>
   <si>
     <t>Verify received category can be created</t>
@@ -401,7 +401,7 @@
     <t>TC-022</t>
   </si>
   <si>
-    <t>Fetch Received Category</t>
+    <t>Fetch received category</t>
   </si>
   <si>
     <t>Verify received category can be retrieved</t>
@@ -416,7 +416,7 @@
     <t>TC-023</t>
   </si>
   <si>
-    <t>Update Received Category</t>
+    <t>Update received category</t>
   </si>
   <si>
     <t>Verify received category can be updated</t>
@@ -428,7 +428,7 @@
     <t>TC-024</t>
   </si>
   <si>
-    <t>Delete Received Category</t>
+    <t>Delete received category</t>
   </si>
   <si>
     <t>Verify received category can be deleted</t>
@@ -437,7 +437,7 @@
     <t>TC-025</t>
   </si>
   <si>
-    <t>Create Debit Transaction</t>
+    <t>Create debit transaction</t>
   </si>
   <si>
     <t>Verify debit transaction can be created</t>
@@ -452,7 +452,7 @@
     <t>TC-026</t>
   </si>
   <si>
-    <t>Fetch Transaction</t>
+    <t>Fetch transactions</t>
   </si>
   <si>
     <t>Verify all transactions can be retrieved</t>
@@ -464,7 +464,7 @@
     <t>TC-027</t>
   </si>
   <si>
-    <t>Update Debit Transaction</t>
+    <t>Update debit transaction</t>
   </si>
   <si>
     <t>Verify debit transaction can be modified</t>
@@ -479,7 +479,7 @@
     <t>TC-028</t>
   </si>
   <si>
-    <t>Delete Debit Transaction</t>
+    <t>Delete debit transaction</t>
   </si>
   <si>
     <t>Verify debit transaction can be removed</t>
@@ -494,7 +494,7 @@
     <t>TC-029</t>
   </si>
   <si>
-    <t>Create Credit Transaction</t>
+    <t>Create credit transaction</t>
   </si>
   <si>
     <t>Verify credit transaction can be created</t>
@@ -506,7 +506,7 @@
     <t>TC-030</t>
   </si>
   <si>
-    <t>Update Credit Transaction</t>
+    <t>Update credit transaction</t>
   </si>
   <si>
     <t>Verify credit transaction can be modified</t>
@@ -518,7 +518,7 @@
     <t>TC-031</t>
   </si>
   <si>
-    <t>Delete Credit Transaction</t>
+    <t>Delete credit transaction</t>
   </si>
   <si>
     <t>Verify credit transaction can be removed</t>
@@ -530,7 +530,7 @@
     <t>TC-032</t>
   </si>
   <si>
-    <t>Create Given Contact Ledger Transaction</t>
+    <t>Create given ledger transaction</t>
   </si>
   <si>
     <t>Verify given transaction can be created for contact ledger</t>
@@ -545,7 +545,7 @@
     <t>TC-033</t>
   </si>
   <si>
-    <t>Create Received Contact Ledger Transaction</t>
+    <t>Create received ledger transaction</t>
   </si>
   <si>
     <t>Verify received transaction can be created for contact ledger</t>
@@ -557,7 +557,7 @@
     <t>TC-034</t>
   </si>
   <si>
-    <t>Delete Given Transaction</t>
+    <t>Delete given ledger transaction</t>
   </si>
   <si>
     <t>Verify given contact ledger transaction can be deleted</t>
@@ -569,7 +569,7 @@
     <t>TC-035</t>
   </si>
   <si>
-    <t>Delete Received Transaction</t>
+    <t>Delete received ledger transaction</t>
   </si>
   <si>
     <t>Verify received contact ledger transaction can be deleted</t>
@@ -578,7 +578,7 @@
     <t>TC-036</t>
   </si>
   <si>
-    <t>Create Contact</t>
+    <t>Create contact</t>
   </si>
   <si>
     <t>Verify contact can be created for contact ledger</t>
@@ -593,7 +593,7 @@
     <t>TC-037</t>
   </si>
   <si>
-    <t>Fetch Contacts</t>
+    <t>Fetch contacts</t>
   </si>
   <si>
     <t>Verify contact details can be retrieved</t>
@@ -605,7 +605,7 @@
     <t>TC-038</t>
   </si>
   <si>
-    <t>Update Contact</t>
+    <t>Update contact</t>
   </si>
   <si>
     <t>Verify contact information can be updated</t>
@@ -620,7 +620,7 @@
     <t>TC-039</t>
   </si>
   <si>
-    <t>Delete Contact</t>
+    <t>Delete contact</t>
   </si>
   <si>
     <t>Verify contact can be deleted from the system</t>
@@ -635,7 +635,7 @@
     <t>TC-040</t>
   </si>
   <si>
-    <t>Table Calculations</t>
+    <t>Validate table totals</t>
   </si>
   <si>
     <t>Verify arithmetic calculations in transaction table are accurate</t>
@@ -647,7 +647,7 @@
     <t>TC-041</t>
   </si>
   <si>
-    <t>Impact Calculation of Created Transaction</t>
+    <t>Validate transaction impact</t>
   </si>
   <si>
     <t>Verify transaction creation impacts summary cards correctly</t>
@@ -1899,7 +1899,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr/>
   <dimension ref="A1:Q42"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>

</xml_diff>